<commit_message>
docs: 확정 스택(Make·Supabase Auth·PostgreSQL)과 어긋난 잔여 표기 정리
기획서 7-2 역할 분담표:
- E 담당 설명의 'n8n 배치 7종' -> 'Make 시나리오 + Python 배치 엔드포인트 7종'

기능명세서_학습플래너.xlsx:
- FR-JOIN-01 세부사항(K15): 'bcrypt 해시로 저장' -> '비밀번호 해싱·저장은 Supabase Auth가 처리'
- FR-STUDY-03 비고(N44): 'Redis 카운터' -> 'PostgreSQL 집계 · Redis는 확장 시'

학습로드맵의 n8n 언급 2건은 '변경 전 -> 변경 후' 이력 표라 의도적으로 유지.
예시_기능명세서 시트는 템플릿 샘플이라 수정 대상 아님.
</commit_message>
<xml_diff>
--- a/기능명세서_학습플래너.xlsx
+++ b/기능명세서_학습플래너.xlsx
@@ -2260,7 +2260,7 @@
     <t xml:space="preserve">이메일, 비밀번호, 닉네임</t>
   </si>
   <si>
-    <t xml:space="preserve">충족하지 못한 조건을 입력 중 실시간으로 표시하고 모두 충족해야 가입 버튼 활성화 / 이메일·닉네임을 포함한 비밀번호와 자주 쓰이는 비밀번호 목록(상위 1만 건)은 거부 / 중복 이메일이면 '이미 가입된 이메일입니다' / bcrypt 해시로 저장</t>
+    <t xml:space="preserve">충족하지 못한 조건을 입력 중 실시간으로 표시하고 모두 충족해야 가입 버튼 활성화 / 이메일·닉네임을 포함한 비밀번호와 자주 쓰이는 비밀번호 목록(상위 1만 건)은 거부 / 중복 이메일이면 '이미 가입된 이메일입니다' / 비밀번호 해싱·저장은 Supabase Auth가 처리</t>
   </si>
   <si>
     <t xml:space="preserve">특수문자 허용 범위를 화면에 명시해야 입력 실패가 줄어듦</t>
@@ -2992,7 +2992,7 @@
     <t xml:space="preserve">카운터 장애 시 이벤트를 큐에 보관하고 복구 후 재집계 / 하루 경계는 사용자 로컬 타임존 기준</t>
   </si>
   <si>
-    <t xml:space="preserve">Redis 카운터</t>
+    <t xml:space="preserve">PostgreSQL 집계 · Redis는 확장 시</t>
   </si>
   <si>
     <t xml:space="preserve">FR-STUDY-04</t>

</xml_diff>

<commit_message>
docs(spec): FR-CONT-06 포스터 정보 추출 Could → Won't
위비티 이용 조건(비영리·원문·포스터 저장 금지)과 충돌해 범위에서 제외. 기능명세서 우선순위·세부 사항·비고와
기획서 MoSCoW 건수(Could 3 / Won't 3)를 함께 고쳤다.
</commit_message>
<xml_diff>
--- a/기능명세서_학습플래너.xlsx
+++ b/기능명세서_학습플래너.xlsx
@@ -6560,21 +6560,29 @@
       </c>
       <c r="J59" s="56" t="inlineStr">
         <is>
-          <t>Could</t>
+          <t>Won't</t>
         </is>
       </c>
       <c r="K59" s="54" t="inlineStr">
         <is>
-          <t>추출 실패 또는 신뢰도 미달이면 미검수 상태로 보관하고 사용자에게 노출하지 않음</t>
-        </is>
-      </c>
-      <c r="L59" s="54" t="n"/>
+          <t>위비티 이용 조건(비영리·원문·포스터 저장 금지, 제목·링크·메타데이터만 사용)과 충돌해 이번 범위에서 제외</t>
+        </is>
+      </c>
+      <c r="L59" s="54" t="inlineStr">
+        <is>
+          <t>포스터 이미지를 받아 저장해야 하는 기능 — 공식 API·제휴로 이미지 사용 허락을 받으면 재검토</t>
+        </is>
+      </c>
       <c r="M59" s="54" t="inlineStr">
         <is>
           <t>관리자</t>
         </is>
       </c>
-      <c r="N59" s="54" t="n"/>
+      <c r="N59" s="54" t="inlineStr">
+        <is>
+          <t>v1.2에서 하향 (Could → Won't, 10-02)</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="45.75" customHeight="1" s="44">
       <c r="A60" s="54" t="inlineStr">

</xml_diff>